<commit_message>
fix: complete new-taipei with all 29 districts
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/excel/02-new-taipei.xlsx
+++ b/data/excel/02-new-taipei.xlsx
@@ -1272,7 +1272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1319,7 +1319,6 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1337,7 +1336,6 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1355,7 +1353,6 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1373,17 +1370,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>中和區</t>
+          <t>三重區</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>環球購物中心</t>
+          <t>三和夜市</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1391,17 +1387,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>中和區</t>
+          <t>三重區</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>南勢角</t>
+          <t>重新路</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1409,17 +1404,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>中和區</t>
+          <t>三重區</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>景安</t>
+          <t>菜寮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1427,17 +1421,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>中和區</t>
+          <t>三重區</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>連城路</t>
+          <t>中山路</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1445,17 +1438,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>永和區</t>
+          <t>中和區</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>樂華夜市</t>
+          <t>環球購物中心</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1463,17 +1455,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>永和區</t>
+          <t>中和區</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>頂溪</t>
+          <t>南勢角</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1481,17 +1472,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>永和區</t>
+          <t>中和區</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>永和路</t>
+          <t>景安</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1499,17 +1489,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>永和區</t>
+          <t>中和區</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>秀朗橋</t>
+          <t>連城路</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1517,17 +1506,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>新莊區</t>
+          <t>永和區</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>新莊廟街</t>
+          <t>樂華夜市</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1535,17 +1523,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>新莊區</t>
+          <t>永和區</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>副都心</t>
+          <t>頂溪</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1553,17 +1540,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>新莊區</t>
+          <t>永和區</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>頭前</t>
+          <t>永和路</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1571,17 +1557,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>新莊區</t>
+          <t>永和區</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>後港路</t>
+          <t>秀朗橋</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1589,17 +1574,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>三重區</t>
+          <t>新莊區</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>三和夜市</t>
+          <t>新莊廟街</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1607,17 +1591,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>三重區</t>
+          <t>新莊區</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>重新路</t>
+          <t>副都心</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1625,17 +1608,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>三重區</t>
+          <t>新莊區</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>菜寮</t>
+          <t>頭前</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1643,17 +1625,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>三重區</t>
+          <t>新莊區</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>中山路</t>
+          <t>後港路</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1661,17 +1642,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>土城區</t>
+          <t>新店區</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>土城老街</t>
+          <t>大坪林</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1679,17 +1659,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>土城區</t>
+          <t>新店區</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>中央路</t>
+          <t>碧潭</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1697,17 +1676,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>土城區</t>
+          <t>新店區</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>金城路</t>
+          <t>北新路</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1715,17 +1693,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>土城區</t>
+          <t>新店區</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>頂埔</t>
+          <t>安康路</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1733,17 +1710,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>新店區</t>
+          <t>樹林區</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>大坪林</t>
+          <t>樹林市區</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1751,17 +1727,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>新店區</t>
+          <t>樹林區</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>碧潭</t>
+          <t>中山路</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1769,17 +1744,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>新店區</t>
+          <t>樹林區</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>北新路</t>
+          <t>自強街</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1787,17 +1761,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>新店區</t>
+          <t>樹林區</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>安康路</t>
+          <t>山佳</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1805,17 +1778,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>淡水區</t>
+          <t>鶯歌區</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>淡水老街</t>
+          <t>鶯歌陶瓷老街</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1823,17 +1795,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>淡水區</t>
+          <t>鶯歌區</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>漁人碼頭</t>
+          <t>鶯歌市區</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1841,17 +1812,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>淡水區</t>
+          <t>鶯歌區</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>淡江大學</t>
+          <t>尖山埔路</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1859,17 +1829,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>淡水區</t>
+          <t>鶯歌區</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>紅毛城</t>
+          <t>南鶯工業區</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1877,17 +1846,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>汐止區</t>
+          <t>三峽區</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>汐止市區</t>
+          <t>三峽老街</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1895,17 +1863,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>汐止區</t>
+          <t>三峽區</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>新台五路</t>
+          <t>清水祖師廟</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1913,17 +1880,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>汐止區</t>
+          <t>三峽區</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>樟樹灣</t>
+          <t>三峽市區</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1931,17 +1897,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>汐止區</t>
+          <t>三峽區</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>遠雄新城</t>
+          <t>鳶山</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1949,17 +1914,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>樹林區</t>
+          <t>淡水區</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>樹林市區</t>
+          <t>淡水老街</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1967,17 +1931,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>樹林區</t>
+          <t>淡水區</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>中山路</t>
+          <t>漁人碼頭</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1985,17 +1948,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>樹林區</t>
+          <t>淡水區</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>自強街</t>
+          <t>淡江大學周邊</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2003,17 +1965,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>樹林區</t>
+          <t>淡水區</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>山佳</t>
+          <t>紅毛城</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2021,17 +1982,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>蘆洲區</t>
+          <t>汐止區</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>蘆洲市區</t>
+          <t>汐止市區</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2039,17 +1999,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>蘆洲區</t>
+          <t>汐止區</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>中山路</t>
+          <t>新台五路</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2057,17 +2016,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>蘆洲區</t>
+          <t>汐止區</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>集賢路</t>
+          <t>樟樹灣</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2075,17 +2033,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>蘆洲區</t>
+          <t>汐止區</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>民族路</t>
+          <t>遠雄新城</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2093,17 +2050,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>林口區</t>
+          <t>瑞芳區</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>林口三井</t>
+          <t>九份老街</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2111,17 +2067,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>林口區</t>
+          <t>瑞芳區</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>長庚醫院周邊</t>
+          <t>瑞芳市區</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2129,17 +2084,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>林口區</t>
+          <t>瑞芳區</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>林口文化三路</t>
+          <t>侯硐貓村</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2147,17 +2101,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>林口區</t>
+          <t>瑞芳區</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>林口市區</t>
+          <t>金瓜石</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2165,17 +2118,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>三峽區</t>
+          <t>土城區</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>三峽老街</t>
+          <t>土城老街</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2183,17 +2135,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>三峽區</t>
+          <t>土城區</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>清水祖師廟</t>
+          <t>中央路</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2201,17 +2152,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>三峽區</t>
+          <t>土城區</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>三峽市區</t>
+          <t>金城路</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2219,17 +2169,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>三峽區</t>
+          <t>土城區</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>鶯歌交界</t>
+          <t>頂埔</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2237,17 +2186,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>鶯歌區</t>
+          <t>蘆洲區</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>鶯歌陶瓷老街</t>
+          <t>蘆洲市區</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2255,17 +2203,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>鶯歌區</t>
+          <t>蘆洲區</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>鶯歌市區</t>
+          <t>中山路</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2273,17 +2220,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>鶯歌區</t>
+          <t>蘆洲區</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>南鶯工業區</t>
+          <t>集賢路</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2291,17 +2237,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>鶯歌區</t>
+          <t>蘆洲區</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>尖山埔路</t>
+          <t>民族路</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2309,17 +2254,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>瑞芳區</t>
+          <t>林口區</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>九份老街</t>
+          <t>林口三井</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2327,17 +2271,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>瑞芳區</t>
+          <t>林口區</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>瑞芳市區</t>
+          <t>長庚醫院周邊</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2345,17 +2288,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>瑞芳區</t>
+          <t>林口區</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>侯硐貓村</t>
+          <t>林口文化三路</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2363,17 +2305,16 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>瑞芳區</t>
+          <t>林口區</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>金瓜石</t>
+          <t>林口市區</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2381,7 +2322,958 @@
           <t>商圈</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>深坑區</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>深坑老街</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>深坑區</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>深坑豆腐街</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>深坑區</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>中山路</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>深坑區</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>北深路</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>石碇區</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>石碇老街</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>石碇區</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>石碇市區</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>石碇區</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>永定溪</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>石碇區</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>溪邊寮</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>坪林區</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>坪林老街</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>坪林區</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>坪林茶博館</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>坪林區</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>北宜路</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>坪林區</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>魚蕨步道</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>三芝區</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>三芝市區</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>三芝區</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>老梅石槽</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>三芝區</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>中山路</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>三芝區</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>新庄子</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>石門區</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>石門老街</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>石門區</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>老梅</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>石門區</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>富貴角燈塔</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>石門區</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>中山路</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>八里區</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>八里老街</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>八里區</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>渡船頭商圈</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>八里區</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>左岸自行車道</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>八里區</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>中山路</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>平溪區</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>平溪老街</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>平溪區</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>十分老街</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>平溪區</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>菁桐老街</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>平溪區</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>天燈商圈</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>雙溪區</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>雙溪市區</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>雙溪區</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>雙溪老街</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>雙溪區</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>中山路</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>雙溪區</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>平林溪</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>貢寮區</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>福隆海水浴場</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>貢寮區</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>貢寮市區</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>貢寮區</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>中山路</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>貢寮區</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>澳底漁港</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>金山區</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>金山老街</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>金山區</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>金山溫泉</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>金山區</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>中山路</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>金山區</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>萬里蟹</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>萬里區</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>萬里市區</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>萬里區</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>野柳地質公園</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>萬里區</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>中山路</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>萬里區</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>萬里蟹</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>烏來區</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>烏來老街</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>烏來區</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>烏來溫泉</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>烏來區</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>信賢步道</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>烏來區</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>福山部落</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>泰山區</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>泰山市區</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>泰山區</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>中山路</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>泰山區</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>貴子坑</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>泰山區</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>明志路</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>五股區</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>五股市區</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>五股區</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>成泰路</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>五股區</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>五股工業區</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>五股區</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>觀音山</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>